<commit_message>
no functionality change; testing large nuclear sensitivity to parameter defaults
</commit_message>
<xml_diff>
--- a/src/technology/nuclear/nuclear.xlsx
+++ b/src/technology/nuclear/nuclear.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhanes\GitHub\tyche\src\technology\nuclear\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B51E09A2-F092-45CD-8D40-F8867D3E5F12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E0AE55-612C-421E-A431-31C22B9B2CFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20775" yWindow="2085" windowWidth="27390" windowHeight="15345" tabRatio="778" activeTab="2" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
+    <workbookView xWindow="1755" yWindow="1920" windowWidth="31095" windowHeight="19035" tabRatio="778" activeTab="4" xr2:uid="{277ED3FD-2B20-4A36-BB03-16AF83BDC75C}"/>
   </bookViews>
   <sheets>
     <sheet name="indices" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">designs!$A$1:$G$92</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">indices!$A$1:$F$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">parameters!$A$1:$G$337</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">parameters!$A$1:$G$651</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -541,7 +541,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -551,6 +551,12 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -576,8 +582,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -20030,7 +20037,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G625" xr:uid="{9375A35C-8A58-4D70-9436-2E641DE51D25}"/>
+  <autoFilter ref="A1:G651" xr:uid="{9375A35C-8A58-4D70-9436-2E641DE51D25}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H162">
     <sortCondition ref="A2:A162"/>
     <sortCondition ref="B2:B162"/>
@@ -20714,7 +20721,7 @@
       <c r="C3">
         <v>1</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>0.8</v>
       </c>
       <c r="E3">
@@ -20834,7 +20841,7 @@
       <c r="C7">
         <v>1000000</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="1">
         <v>22000</v>
       </c>
       <c r="E7">
@@ -20924,7 +20931,7 @@
       <c r="C10">
         <v>1</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="1">
         <v>0.8</v>
       </c>
       <c r="E10">

</xml_diff>